<commit_message>
fix(psdash,kmplot,pkgtransfer): sync release fixes and add pkgtransfe...
Bump kmplot to 1.2.6: _kmplot_risktable.ado adds TOPTimeaxis to
xaxis(1 2) the number-at-risk table above a horizontal separator and
raise its label size from vsmall to small, matching kmplot.ado,
kmplot.sthlp, and README.md. Bump psdash to 1.6.7 across its .ado
helpers with README synced. Add pkgtransfer/README.md and new
demo/console_*.md walkthroughs plus demo/demo_pkgtransfer.do. Add
kmplot/qa/test_kmplot_v126.do regression coverage and update
qa/README.md and qa/run_all.do to include it. Regenerate demo
artifacts across codescan, finegray, iivw, and kmplot
(codescan_results.xlsx, prevalence_chart.png, finegray_cif.png,
iivw_psdash_dashboard.png, iivw_psdash_final_weights.png,
iivw_reporting_exports.xlsx, iivw_results.xlsx, and the km_*.png set)
to reflect current output. Update the root README.md version/date
badges for psdash and kmplot.
</commit_message>
<xml_diff>
--- a/psdash/demo/psdash_report.xlsx
+++ b/psdash/demo/psdash_report.xlsx
@@ -2727,7 +2727,7 @@
         <v>0.0133601195235551</v>
       </c>
       <c r="J3" s="53">
-        <v>1.0070175475116769</v>
+        <v>1.006001716637021</v>
       </c>
       <c r="K3" s="54">
         <v>0.050854877187559502</v>
@@ -2744,10 +2744,10 @@
         <v>0.37751004016064249</v>
       </c>
       <c r="D4" s="57">
-        <v>0.43031695072119203</v>
+        <v>0.43094226089634691</v>
       </c>
       <c r="E4" s="58">
-        <v>1.028603636082803</v>
+        <v>1.030876909735525</v>
       </c>
       <c r="F4" s="59">
         <v>0.2105117384237494</v>
@@ -2759,10 +2759,10 @@
         <v>0.52192770278459788</v>
       </c>
       <c r="I4" s="62">
-        <v>0.0011499000107072</v>
+        <v>0.0011515709748091</v>
       </c>
       <c r="J4" s="63">
-        <v>0.99769489764372021</v>
+        <v>0.99989986119304719</v>
       </c>
       <c r="K4" s="64">
         <v>0.00056253291872829995</v>
@@ -2797,7 +2797,7 @@
         <v>0.013785947066266801</v>
       </c>
       <c r="J5" s="73">
-        <v>1.0726598498761111</v>
+        <v>1.0715778022035549</v>
       </c>
       <c r="K5" s="74">
         <v>0.0447537937716748</v>
@@ -2832,7 +2832,7 @@
         <v>0.0182255436196882</v>
       </c>
       <c r="J6" s="83">
-        <v>1.0508027094953121</v>
+        <v>1.049742710254866</v>
       </c>
       <c r="K6" s="84">
         <v>0.093744814098041002</v>
@@ -2867,7 +2867,7 @@
         <v>0.047032989657052</v>
       </c>
       <c r="J7" s="93">
-        <v>0.99087308437154431</v>
+        <v>0.98987353925491961</v>
       </c>
       <c r="K7" s="94">
         <v>0.0376989109603907</v>

</xml_diff>

<commit_message>
fix(psdash): 1.7.3 support bounds, binary detection, display and labels
Common-support bounds are held in scalars, so the observation that
defines a bound is no longer counted outside it (overlap, support,
qtrim, generate(), multi-group, longitudinal helper). Two-valued
non-integer covariates are treated as binary. Balance table cells no
longer fuse with negative values; ks adds KS Adj columns matching
r(max_ks_adj). matched no longer needs a propensity score; strategies()
refuses undefined att/ate weights. The multi-group Love plot names
contrasts by value label and shows raw and adjusted SMDs; count axes
print whole numbers; labels are drawn verbatim via _psdash_label_text.
Help corrects the cobalt denominator claim. Demo regenerated with
white_tableau. New suite qa/test_v173_audit_regressions.do (18 tests).
</commit_message>
<xml_diff>
--- a/psdash/demo/psdash_report.xlsx
+++ b/psdash/demo/psdash_report.xlsx
@@ -2497,7 +2497,7 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
+      <c r="B1" s="0"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
@@ -2652,16 +2652,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="0"/>
-      <c r="C1" s="0"/>
-      <c r="D1" s="0"/>
-      <c r="E1" s="0"/>
-      <c r="F1" s="0"/>
-      <c r="G1" s="0"/>
-      <c r="H1" s="0"/>
-      <c r="I1" s="0"/>
-      <c r="J1" s="0"/>
-      <c r="K1" s="0"/>
+      <c r="A1" s="22" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="34" t="s">
@@ -2718,19 +2711,19 @@
         <v>0.20893009424266951</v>
       </c>
       <c r="G3" s="50">
-        <v>54.599767364271919</v>
+        <v>54.599767364271912</v>
       </c>
       <c r="H3" s="51">
         <v>54.447923722146967</v>
       </c>
       <c r="I3" s="52">
-        <v>0.0133601195235551</v>
+        <v>0.0133601195235545</v>
       </c>
       <c r="J3" s="53">
         <v>1.006001716637021</v>
       </c>
       <c r="K3" s="54">
-        <v>0.050854877187559502</v>
+        <v>0.050854877187559197</v>
       </c>
     </row>
     <row r="4">
@@ -2765,7 +2758,7 @@
         <v>0.99989986119304719</v>
       </c>
       <c r="K4" s="64">
-        <v>0.00056253291872819999</v>
+        <v>0.00056253291872879999</v>
       </c>
     </row>
     <row r="5">
@@ -2788,13 +2781,13 @@
         <v>0.098178558152756307</v>
       </c>
       <c r="G5" s="70">
-        <v>26.858463466152841</v>
+        <v>26.858463466152831</v>
       </c>
       <c r="H5" s="71">
         <v>26.790461036418598</v>
       </c>
       <c r="I5" s="72">
-        <v>0.013785947066266801</v>
+        <v>0.0137859470662647</v>
       </c>
       <c r="J5" s="73">
         <v>1.0715778022035549</v>
@@ -2835,7 +2828,7 @@
         <v>1.049742710254866</v>
       </c>
       <c r="K6" s="84">
-        <v>0.093744814098041002</v>
+        <v>0.093744814098040793</v>
       </c>
     </row>
     <row r="7">
@@ -2858,25 +2851,22 @@
         <v>0.038753926777892002</v>
       </c>
       <c r="G7" s="90">
-        <v>201.3617161279218</v>
+        <v>201.36171612792171</v>
       </c>
       <c r="H7" s="91">
         <v>199.5066106886371</v>
       </c>
       <c r="I7" s="92">
-        <v>0.047032989657052</v>
+        <v>0.047032989657049801</v>
       </c>
       <c r="J7" s="93">
         <v>0.98987353925491961</v>
       </c>
       <c r="K7" s="94">
-        <v>0.0376989109603907</v>
+        <v>0.037698910960390797</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
-  </mergeCells>
 </worksheet>
 </file>
 
@@ -2890,7 +2880,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="0"/>
+      <c r="A1" s="97" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="99" t="s">
@@ -3053,9 +3045,6 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
-  </mergeCells>
 </worksheet>
 </file>
 
@@ -3069,7 +3058,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="0"/>
+      <c r="A1" s="122" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="124" t="s">
@@ -3168,9 +3159,6 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
-  </mergeCells>
 </worksheet>
 </file>
 
@@ -3184,7 +3172,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="0"/>
+      <c r="A1" s="138" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="140" t="s">
@@ -3275,8 +3265,5 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
-  </mergeCells>
 </worksheet>
 </file>
</xml_diff>